<commit_message>
Add SpaceX free-float bridge and Tesla related-party check
</commit_message>
<xml_diff>
--- a/25-ipo-six-month-price-action/ipo_six_month_price_action_model.xlsx
+++ b/25-ipo-six-month-price-action/ipo_six_month_price_action_model.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,6 +557,23 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>Fast-entry and low-float index weighting rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tesla 10-Q</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1318605/000162828026026673/tsla-20260331.htm</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Tesla's March 2026 SpaceX common-stock investment and related-party Megapack transactions.</t>
         </is>
       </c>
     </row>
@@ -6577,7 +6594,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Elon Musk</t>
+          <t>Elon Musk; Tesla small economic interest</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -6591,12 +6608,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Musk and directors/officers dominate voting control; 13F data is future monitoring only.</t>
+          <t>Musk and directors/officers dominate voting control. Tesla 10-Q says Tesla invested $2.00B in SpaceX common stock, less than 1% ownership; estimated at about 0.11% of SpaceX basic shares at the IPO price. 13F data is future monitoring only.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>S-1/A</t>
+          <t>S-1/A; Tesla 10-Q</t>
         </is>
       </c>
       <c r="H2" t="n">

</xml_diff>